<commit_message>
Feature: Switch Excel export to ExcelJS to support embedding the college logo directly from the browser
</commit_message>
<xml_diff>
--- a/project docs/SK_College_Admission_Report_2026.xlsx
+++ b/project docs/SK_College_Admission_Report_2026.xlsx
@@ -768,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:J17"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -780,7 +780,6 @@
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
     <col min="10" max="10" width="40.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
@@ -814,9 +813,6 @@
       <c r="J1" s="4" t="str">
         <v/>
       </c>
-      <c r="K1" s="4" t="str">
-        <v/>
-      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="5" t="str">
@@ -849,9 +845,6 @@
       <c r="J2" s="6" t="str">
         <v/>
       </c>
-      <c r="K2" s="6" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="7" t="str">
@@ -884,9 +877,6 @@
       <c r="J3" s="7" t="str">
         <v/>
       </c>
-      <c r="K3" s="7" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="str">
@@ -919,9 +909,6 @@
       <c r="J4" s="8" t="str">
         <v/>
       </c>
-      <c r="K4" s="8" t="str">
-        <v/>
-      </c>
     </row>
     <row r="5" ht="8" customHeight="1">
       <c r="A5" s="9" t="str">
@@ -952,9 +939,6 @@
         <v/>
       </c>
       <c r="J5" s="10" t="str">
-        <v/>
-      </c>
-      <c r="K5" s="10" t="str">
         <v/>
       </c>
     </row>
@@ -989,13 +973,10 @@
       <c r="J6" s="12" t="str">
         <v/>
       </c>
-      <c r="K6" s="12" t="str">
-        <v/>
-      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="13" t="str">
-        <v>Date of Printing: 25 April 2026 | 02:15 pm</v>
+        <v>Date of Printing: 25 April 2026 | 02:35 pm</v>
       </c>
       <c r="B7" s="13" t="str">
         <v/>
@@ -1022,9 +1003,6 @@
         <v/>
       </c>
       <c r="J7" s="13" t="str">
-        <v/>
-      </c>
-      <c r="K7" s="13" t="str">
         <v/>
       </c>
     </row>
@@ -1059,9 +1037,6 @@
       <c r="J8" s="15" t="str">
         <v>Address</v>
       </c>
-      <c r="K8" s="15" t="str">
-        <v>Application ID</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="16">
@@ -1093,9 +1068,6 @@
       </c>
       <c r="J9" s="18" t="str">
         <v>Vootapalli</v>
-      </c>
-      <c r="K9" s="16" t="str">
-        <v>71932711</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -1131,9 +1103,6 @@
 Gantyada 
 Vizianagaram</v>
       </c>
-      <c r="K10" s="19" t="str">
-        <v>ADA3B10A</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="16">
@@ -1166,9 +1135,6 @@
       <c r="J11" s="18" t="str">
         <v>9948057328</v>
       </c>
-      <c r="K11" s="16" t="str">
-        <v>1EBD4B76</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="19">
@@ -1201,9 +1167,6 @@
       <c r="J12" s="20" t="str">
         <v>Gallavilli</v>
       </c>
-      <c r="K12" s="19" t="str">
-        <v>D46CF2D3</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="16">
@@ -1236,9 +1199,6 @@
       <c r="J13" s="18" t="str">
         <v>Pedakada (v), Dattirajeru (m), vizianagaram (d), Andhra Pradesh (s)</v>
       </c>
-      <c r="K13" s="16" t="str">
-        <v>B0B7A52E</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="19">
@@ -1271,9 +1231,6 @@
       <c r="J14" s="20" t="str">
         <v>Gantyada(mandalam); Vizianagaram (DIST);madhnapuram(village)</v>
       </c>
-      <c r="K14" s="19" t="str">
-        <v>7DD12B06</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="str">
@@ -1306,9 +1263,6 @@
       <c r="J15" s="22" t="str">
         <v/>
       </c>
-      <c r="K15" s="22" t="str">
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
@@ -1339,9 +1293,6 @@
         <v/>
       </c>
       <c r="J16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="K16" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -1376,24 +1327,21 @@
       <c r="J17" s="23" t="str">
         <v/>
       </c>
-      <c r="K17" s="23" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A7:K7"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A17:J17"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(nav): add nirf rank to navigation menu and update roadmap state
</commit_message>
<xml_diff>
--- a/project docs/SK_College_Admission_Report_2026.xlsx
+++ b/project docs/SK_College_Admission_Report_2026.xlsx
@@ -7,14 +7,14 @@
     <sheet sheetId="1" name="Admission Report" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Admission Report'!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Admission Report'!$1:$7</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>S.K. DEGREE COLLEGE &amp; PG COLLEGE</t>
   </si>
@@ -22,16 +22,13 @@
     <t>Affiliated to Andhra University | Established in 2005</t>
   </si>
   <si>
-    <t>School Nagar, Ayyannapet Junction, Vizianagaram, Andhra Pradesh</t>
-  </si>
-  <si>
     <t>Ph: 94412 53163 | Email: arunodayaes@yahoo.com | www.skdegreecollege.com</t>
   </si>
   <si>
     <t>ONLINE APPLICATION LIST – ADMISSIONS 2026-27</t>
   </si>
   <si>
-    <t>Date of Printing: 25 April 2026 | 02:44 pm</t>
+    <t>Date of Printing: 25 April 2026 | 02:52 pm</t>
   </si>
   <si>
     <t>S.No</t>
@@ -111,21 +108,6 @@
 Vizianagaram</t>
   </si>
   <si>
-    <t>Srinivasarao Bankuru</t>
-  </si>
-  <si>
-    <t>naveenkumarbankuru04@gmail.com</t>
-  </si>
-  <si>
-    <t>7207943787</t>
-  </si>
-  <si>
-    <t>mpc</t>
-  </si>
-  <si>
-    <t>9948057328</t>
-  </si>
-  <si>
     <t xml:space="preserve">V sailaja </t>
   </si>
   <si>
@@ -171,7 +153,7 @@
     <t>Gantyada(mandalam); Vizianagaram (DIST);madhnapuram(village)</t>
   </si>
   <si>
-    <t>Total Applications Received: 6</t>
+    <t>Total Applications Received: 5</t>
   </si>
   <si>
     <t>This is a computer-generated report from the S.K. Degree College online admission portal. For queries, contact the college administration.</t>
@@ -181,7 +163,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -199,11 +181,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF1B5E20"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -327,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -338,38 +315,35 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -393,7 +367,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -758,7 +732,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -773,10 +747,10 @@
   </cols>
   <sheetData>
     <row r="1" ht="55" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -800,7 +774,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -814,10 +788,8 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>3</v>
-      </c>
+    <row r="4" ht="8" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -828,8 +800,10 @@
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
     </row>
-    <row r="5" ht="8" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
+    <row r="5" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>3</v>
+      </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -840,7 +814,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
     </row>
-    <row r="6" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
@@ -854,247 +828,215 @@
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
     </row>
-    <row r="7" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-    </row>
-    <row r="8" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>6</v>
       </c>
+      <c r="C7" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>1</v>
+      </c>
       <c r="B8" s="8" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>13</v>
+        <v>20</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
-        <v>1</v>
-      </c>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="11">
+        <v>2</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="D9" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>3</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>4</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>5</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="9" t="s">
+      <c r="G12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
-        <v>2</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="9">
-        <v>3</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="9" t="s">
+      <c r="I12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
-        <v>4</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="J12" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="9">
-        <v>5</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="J12" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J13" s="11" t="s">
+    </row>
+    <row r="13" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
-        <v>6</v>
-      </c>
-      <c r="B14" s="12" t="s">
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
         <v>46</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>51</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
@@ -1106,31 +1048,16 @@
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-    </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B1:J1"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A17:J17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>